<commit_message>
Modified excel-file for Lab_1D
</commit_message>
<xml_diff>
--- a/Labs.xlsx
+++ b/Labs.xlsx
@@ -5,59 +5,105 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Documenten\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1KHAI\2 semester\ASPPR-Labs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91356B7C-1687-4C00-8457-F7EBBF945DDF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C12BA12-6F4C-49EC-8AC1-495E04EC2929}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="1" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
   </bookViews>
   <sheets>
     <sheet name="PartC" sheetId="1" r:id="rId1"/>
+    <sheet name="PractD" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">PartC!$B$1:$E$1</definedName>
+    <definedName name="solver_adj" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
     <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
+    <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_drv" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">PartC!$B$1:$E$1</definedName>
+    <definedName name="solver_lhs1" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">PartC!$F$3</definedName>
+    <definedName name="solver_lhs2" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
     <definedName name="solver_lhs3" localSheetId="0" hidden="1">PartC!$F$4</definedName>
+    <definedName name="solver_lhs3" localSheetId="1" hidden="1">PractD!$F$3</definedName>
     <definedName name="solver_lhs4" localSheetId="0" hidden="1">PartC!$F$5</definedName>
+    <definedName name="solver_lhs4" localSheetId="1" hidden="1">PractD!$F$4</definedName>
     <definedName name="solver_lhs5" localSheetId="0" hidden="1">PartC!$F$6</definedName>
+    <definedName name="solver_lhs5" localSheetId="1" hidden="1">PractD!$F$5</definedName>
+    <definedName name="solver_lhs6" localSheetId="1" hidden="1">PractD!$F$6</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_mip" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
+    <definedName name="solver_mni" localSheetId="1" hidden="1">30</definedName>
     <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
+    <definedName name="solver_mrt" localSheetId="1" hidden="1">0.075</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_msl" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_nod" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">5</definedName>
+    <definedName name="solver_num" localSheetId="1" hidden="1">6</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">PartC!$G$7</definedName>
+    <definedName name="solver_opt" localSheetId="1" hidden="1">PractD!$G$7</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
+    <definedName name="solver_pre" localSheetId="1" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rbv" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rel1" localSheetId="1" hidden="1">4</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rel2" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel3" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel4" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel4" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel5" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rel6" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_rhs1" localSheetId="1" hidden="1">"ціле"</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">PartC!$G$3</definedName>
+    <definedName name="solver_rhs2" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_rhs3" localSheetId="0" hidden="1">PartC!$G$4</definedName>
+    <definedName name="solver_rhs3" localSheetId="1" hidden="1">PractD!$G$3</definedName>
     <definedName name="solver_rhs4" localSheetId="0" hidden="1">PartC!$G$5</definedName>
+    <definedName name="solver_rhs4" localSheetId="1" hidden="1">PractD!$G$4</definedName>
     <definedName name="solver_rhs5" localSheetId="0" hidden="1">PartC!$G$6</definedName>
+    <definedName name="solver_rhs5" localSheetId="1" hidden="1">PractD!$G$5</definedName>
+    <definedName name="solver_rhs6" localSheetId="1" hidden="1">PractD!$G$6</definedName>
     <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_rsd" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_ssz" localSheetId="0" hidden="1">100</definedName>
+    <definedName name="solver_ssz" localSheetId="1" hidden="1">100</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
     <definedName name="solver_tol" localSheetId="0" hidden="1">0.01</definedName>
+    <definedName name="solver_tol" localSheetId="1" hidden="1">0.01</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_typ" localSheetId="1" hidden="1">2</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -75,7 +121,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
   <si>
     <t>x1=</t>
   </si>
@@ -120,6 +166,9 @@
   </si>
   <si>
     <t>Вхідна симплекс-таблиця</t>
+  </si>
+  <si>
+    <t>y4</t>
   </si>
 </sst>
 </file>
@@ -221,7 +270,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -253,6 +302,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -854,4 +909,294 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B038338A-BE43-46BF-B04F-E653862170B8}">
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" s="2">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>0</v>
+      </c>
+      <c r="B3" s="6">
+        <v>1</v>
+      </c>
+      <c r="C3" s="6">
+        <v>-1</v>
+      </c>
+      <c r="D3" s="6">
+        <v>1</v>
+      </c>
+      <c r="E3" s="6">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5">
+        <f>SUMPRODUCT(B3:E3,$B$1:$E$1)</f>
+        <v>-2</v>
+      </c>
+      <c r="G3" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="6">
+        <v>1</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6">
+        <v>-1</v>
+      </c>
+      <c r="F4" s="5">
+        <f t="shared" ref="F4:F6" si="0">SUMPRODUCT(B4:E4,$B$1:$E$1)</f>
+        <v>2</v>
+      </c>
+      <c r="G4" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="6">
+        <v>-1</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G5" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="6">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6">
+        <v>-1</v>
+      </c>
+      <c r="E6" s="6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G6" s="9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="7">
+        <v>-1</v>
+      </c>
+      <c r="C7" s="7">
+        <v>-3</v>
+      </c>
+      <c r="D7" s="7">
+        <v>5</v>
+      </c>
+      <c r="E7" s="7">
+        <v>4</v>
+      </c>
+      <c r="F7" s="4"/>
+      <c r="G7" s="8">
+        <f>SUMPRODUCT(B7:E7,B1:E1)</f>
+        <v>-6</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4">
+        <v>-1</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+      <c r="F12" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="4">
+        <v>1</v>
+      </c>
+      <c r="C13" s="4">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4">
+        <v>-1</v>
+      </c>
+      <c r="F13" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="4">
+        <v>-1</v>
+      </c>
+      <c r="C14" s="4">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="4">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4">
+        <v>1</v>
+      </c>
+      <c r="D15" s="4">
+        <v>-1</v>
+      </c>
+      <c r="E15" s="4">
+        <v>1</v>
+      </c>
+      <c r="F15" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="4">
+        <v>-1</v>
+      </c>
+      <c r="C16" s="4">
+        <v>-3</v>
+      </c>
+      <c r="D16" s="4">
+        <v>5</v>
+      </c>
+      <c r="E16" s="4">
+        <v>4</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:F10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Change excel file: add lab_2 list
</commit_message>
<xml_diff>
--- a/Labs.xlsx
+++ b/Labs.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1KHAI\2 semester\ASPPR-Labs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C12BA12-6F4C-49EC-8AC1-495E04EC2929}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B98EC1B-9831-45C0-A815-DABE91ABFC12}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="1" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="2" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
   </bookViews>
   <sheets>
     <sheet name="PartC" sheetId="1" r:id="rId1"/>
     <sheet name="PractD" sheetId="2" r:id="rId2"/>
+    <sheet name="Lab_2" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="solver_adj" localSheetId="0" hidden="1">PartC!$B$1:$E$1</definedName>
@@ -121,7 +122,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="23">
   <si>
     <t>x1=</t>
   </si>
@@ -169,6 +170,27 @@
   </si>
   <si>
     <t>y4</t>
+  </si>
+  <si>
+    <t>Формулювання двоїстої задачі (Lab_2)</t>
+  </si>
+  <si>
+    <t>Вхідна симплекс-таблиця (Lab_1B)</t>
+  </si>
+  <si>
+    <t>Формулювання прямої задачі (Lab_2)</t>
+  </si>
+  <si>
+    <t>W=2u1-u2 -&gt; min</t>
+  </si>
+  <si>
+    <t>v1=3u1+u2&gt;=2</t>
+  </si>
+  <si>
+    <t>v2=-u1-2u2&gt;=1</t>
+  </si>
+  <si>
+    <t>u2&gt;=0</t>
   </si>
 </sst>
 </file>
@@ -270,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -301,14 +323,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -325,6 +350,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>305098</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>181080</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0C144164-3F74-44E7-B874-A052F4C3963C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1714500"/>
+          <a:ext cx="2133898" cy="752580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -777,14 +851,14 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
@@ -1094,7 +1168,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="4">
@@ -1114,7 +1188,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B13" s="4">
@@ -1134,7 +1208,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B14" s="4">
@@ -1154,7 +1228,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B15" s="4">
@@ -1174,7 +1248,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B16" s="4">
@@ -1199,4 +1273,174 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99A1F516-7B01-4ABB-AFB8-30960710DAFD}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4">
+        <v>-1</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4">
+        <v>-1</v>
+      </c>
+      <c r="F4" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="4">
+        <v>-1</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4">
+        <v>1</v>
+      </c>
+      <c r="F5" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4">
+        <v>-1</v>
+      </c>
+      <c r="E6" s="4">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-1</v>
+      </c>
+      <c r="C7" s="4">
+        <v>-3</v>
+      </c>
+      <c r="D7" s="4">
+        <v>5</v>
+      </c>
+      <c r="E7" s="4">
+        <v>4</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Checking the solution of problem option #2 in Excel
</commit_message>
<xml_diff>
--- a/Labs.xlsx
+++ b/Labs.xlsx
@@ -8,30 +8,39 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1KHAI\2 semester\ASPPR-Labs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B98EC1B-9831-45C0-A815-DABE91ABFC12}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31ACE702-6FED-4888-806A-79D76982FAF1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="2" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="3" xr2:uid="{65BE1558-4BAB-4378-8996-D166A0893C9D}"/>
   </bookViews>
   <sheets>
     <sheet name="PartC" sheetId="1" r:id="rId1"/>
     <sheet name="PractD" sheetId="2" r:id="rId2"/>
     <sheet name="Lab_2" sheetId="3" r:id="rId3"/>
+    <sheet name="Lab_5" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="solver_adj" localSheetId="3" hidden="1">Lab_5!$C$3:$F$5</definedName>
     <definedName name="solver_adj" localSheetId="0" hidden="1">PartC!$B$1:$E$1</definedName>
     <definedName name="solver_adj" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
+    <definedName name="solver_cvg" localSheetId="3" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
     <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_drv" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_drv" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_eng" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_eng" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_est" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_est" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_itr" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="3" hidden="1">Lab_5!$C$6:$F$6</definedName>
     <definedName name="solver_lhs1" localSheetId="0" hidden="1">PartC!$B$1:$E$1</definedName>
     <definedName name="solver_lhs1" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
+    <definedName name="solver_lhs2" localSheetId="3" hidden="1">Lab_5!$G$3:$G$5</definedName>
     <definedName name="solver_lhs2" localSheetId="0" hidden="1">PartC!$F$3</definedName>
     <definedName name="solver_lhs2" localSheetId="1" hidden="1">PractD!$B$1:$E$1</definedName>
     <definedName name="solver_lhs3" localSheetId="0" hidden="1">PartC!$F$4</definedName>
@@ -41,30 +50,43 @@
     <definedName name="solver_lhs5" localSheetId="0" hidden="1">PartC!$F$6</definedName>
     <definedName name="solver_lhs5" localSheetId="1" hidden="1">PractD!$F$5</definedName>
     <definedName name="solver_lhs6" localSheetId="1" hidden="1">PractD!$F$6</definedName>
+    <definedName name="solver_mip" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_mip" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="3" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
     <definedName name="solver_mni" localSheetId="1" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="3" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
     <definedName name="solver_mrt" localSheetId="1" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_msl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_neg" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_neg" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_nod" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_nod" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">5</definedName>
     <definedName name="solver_num" localSheetId="1" hidden="1">6</definedName>
+    <definedName name="solver_nwt" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_nwt" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="3" hidden="1">Lab_5!$B$12</definedName>
     <definedName name="solver_opt" localSheetId="0" hidden="1">PartC!$G$7</definedName>
     <definedName name="solver_opt" localSheetId="1" hidden="1">PractD!$G$7</definedName>
+    <definedName name="solver_pre" localSheetId="3" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
     <definedName name="solver_pre" localSheetId="1" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rbv" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_rel1" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_rel1" localSheetId="1" hidden="1">4</definedName>
+    <definedName name="solver_rel2" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rel2" localSheetId="1" hidden="1">3</definedName>
     <definedName name="solver_rel3" localSheetId="0" hidden="1">1</definedName>
@@ -74,8 +96,10 @@
     <definedName name="solver_rel5" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel5" localSheetId="1" hidden="1">1</definedName>
     <definedName name="solver_rel6" localSheetId="1" hidden="1">1</definedName>
+    <definedName name="solver_rhs1" localSheetId="3" hidden="1">Lab_5!$C$2:$F$2</definedName>
     <definedName name="solver_rhs1" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_rhs1" localSheetId="1" hidden="1">"ціле"</definedName>
+    <definedName name="solver_rhs2" localSheetId="3" hidden="1">Lab_5!$B$3:$B$5</definedName>
     <definedName name="solver_rhs2" localSheetId="0" hidden="1">PartC!$G$3</definedName>
     <definedName name="solver_rhs2" localSheetId="1" hidden="1">0</definedName>
     <definedName name="solver_rhs3" localSheetId="0" hidden="1">PartC!$G$4</definedName>
@@ -85,24 +109,34 @@
     <definedName name="solver_rhs5" localSheetId="0" hidden="1">PartC!$G$6</definedName>
     <definedName name="solver_rhs5" localSheetId="1" hidden="1">PractD!$G$5</definedName>
     <definedName name="solver_rhs6" localSheetId="1" hidden="1">PractD!$G$6</definedName>
+    <definedName name="solver_rlx" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_rlx" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_rsd" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="3" hidden="1">1</definedName>
     <definedName name="solver_scl" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_scl" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_sho" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_sho" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="3" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="0" hidden="1">100</definedName>
     <definedName name="solver_ssz" localSheetId="1" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="3" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_tim" localSheetId="1" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="3" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="0" hidden="1">0.01</definedName>
     <definedName name="solver_tol" localSheetId="1" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="3" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_typ" localSheetId="1" hidden="1">2</definedName>
+    <definedName name="solver_val" localSheetId="3" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
     <definedName name="solver_val" localSheetId="1" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="3" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
     <definedName name="solver_ver" localSheetId="1" hidden="1">3</definedName>
   </definedNames>
@@ -122,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="32">
   <si>
     <t>x1=</t>
   </si>
@@ -191,13 +225,40 @@
   </si>
   <si>
     <t>u2&gt;=0</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>C=</t>
+  </si>
+  <si>
+    <t>S=</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,8 +293,23 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -261,6 +337,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -292,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -326,14 +426,39 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,14 +976,14 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
@@ -1140,14 +1265,14 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
@@ -1281,14 +1406,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
@@ -1409,10 +1534,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="15" t="s">
+      <c r="H9" s="14" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1443,4 +1568,189 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA1C3001-4B4A-4038-9F62-4FBBAA13DA25}">
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C1" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C2" s="19">
+        <v>115</v>
+      </c>
+      <c r="D2" s="19">
+        <v>90</v>
+      </c>
+      <c r="E2" s="19">
+        <v>125</v>
+      </c>
+      <c r="F2" s="19">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="20">
+        <v>130</v>
+      </c>
+      <c r="C3" s="22">
+        <v>115</v>
+      </c>
+      <c r="D3" s="22">
+        <v>10</v>
+      </c>
+      <c r="E3" s="22">
+        <v>5</v>
+      </c>
+      <c r="F3" s="22">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <f>SUM(C3:F3)</f>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="20">
+        <v>80</v>
+      </c>
+      <c r="C4" s="22">
+        <v>0</v>
+      </c>
+      <c r="D4" s="22">
+        <v>80</v>
+      </c>
+      <c r="E4" s="22">
+        <v>0</v>
+      </c>
+      <c r="F4" s="22">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <f t="shared" ref="G4:G5" si="0">SUM(C4:F4)</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="20">
+        <v>195</v>
+      </c>
+      <c r="C5" s="22">
+        <v>0</v>
+      </c>
+      <c r="D5" s="22">
+        <v>0</v>
+      </c>
+      <c r="E5" s="22">
+        <v>120</v>
+      </c>
+      <c r="F5" s="22">
+        <v>75</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C6" s="17">
+        <f>SUM(C3:C5)</f>
+        <v>115</v>
+      </c>
+      <c r="D6" s="17">
+        <f t="shared" ref="D6:F6" si="1">SUM(D3:D5)</f>
+        <v>90</v>
+      </c>
+      <c r="E6" s="17">
+        <f t="shared" si="1"/>
+        <v>125</v>
+      </c>
+      <c r="F6" s="17">
+        <f t="shared" si="1"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="21">
+        <v>5</v>
+      </c>
+      <c r="C8" s="13">
+        <v>7</v>
+      </c>
+      <c r="D8" s="13">
+        <v>8</v>
+      </c>
+      <c r="E8" s="13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="21">
+        <v>6</v>
+      </c>
+      <c r="C9" s="13">
+        <v>2</v>
+      </c>
+      <c r="D9" s="13">
+        <v>4</v>
+      </c>
+      <c r="E9" s="13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="21">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13">
+        <v>3</v>
+      </c>
+      <c r="D10" s="13">
+        <v>3</v>
+      </c>
+      <c r="E10" s="13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="24">
+        <f>SUMPRODUCT(C3:F5, B8:E10)</f>
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="23"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>